<commit_message>
Atualiza base de estoque (39.510 produtos) e dados de execucao para Vercel
</commit_message>
<xml_diff>
--- a/plano_compra_filtro3.xlsx
+++ b/plano_compra_filtro3.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="68">
   <si>
     <t>Codigo</t>
   </si>
@@ -31,6 +31,78 @@
     <t>Quantidade</t>
   </si>
   <si>
+    <t>4958</t>
+  </si>
+  <si>
+    <t>3239 - TERMOMETRO CULINARIO</t>
+  </si>
+  <si>
+    <t>90251199</t>
+  </si>
+  <si>
+    <t>UN</t>
+  </si>
+  <si>
+    <t>5088</t>
+  </si>
+  <si>
+    <t>602 MOCHILA</t>
+  </si>
+  <si>
+    <t>52010020</t>
+  </si>
+  <si>
+    <t>9313</t>
+  </si>
+  <si>
+    <t>BORRACHA STICH</t>
+  </si>
+  <si>
+    <t>40030000</t>
+  </si>
+  <si>
+    <t>9354</t>
+  </si>
+  <si>
+    <t>1353 CANETA</t>
+  </si>
+  <si>
+    <t>9357</t>
+  </si>
+  <si>
+    <t>2205-6 BORRACHA</t>
+  </si>
+  <si>
+    <t>9358</t>
+  </si>
+  <si>
+    <t>EL-4 KIT DE COLORIR INFANTIL</t>
+  </si>
+  <si>
+    <t>48021000</t>
+  </si>
+  <si>
+    <t>9373</t>
+  </si>
+  <si>
+    <t>EL-4-1 KIT DE COLORIR INFANTIL</t>
+  </si>
+  <si>
+    <t>9379</t>
+  </si>
+  <si>
+    <t>FAN-6 PASCOA COM CANETA APUARELA PAPEL MASCARA ANIMAL SERIE</t>
+  </si>
+  <si>
+    <t>9446</t>
+  </si>
+  <si>
+    <t>MAQUINA DE ALGODAO DOCE</t>
+  </si>
+  <si>
+    <t>85141900</t>
+  </si>
+  <si>
     <t>10161</t>
   </si>
   <si>
@@ -40,18 +112,6 @@
     <t>39231010</t>
   </si>
   <si>
-    <t>UN</t>
-  </si>
-  <si>
-    <t>10310</t>
-  </si>
-  <si>
-    <t>TINTA SPRAY KOLORE FASHION 125ML 24 UNID CORES VARIADAS</t>
-  </si>
-  <si>
-    <t>32139000</t>
-  </si>
-  <si>
     <t>12362</t>
   </si>
   <si>
@@ -61,6 +121,33 @@
     <t>85065010</t>
   </si>
   <si>
+    <t>15017</t>
+  </si>
+  <si>
+    <t>964 BOBBIE GOODS</t>
+  </si>
+  <si>
+    <t>49011000</t>
+  </si>
+  <si>
+    <t>18427</t>
+  </si>
+  <si>
+    <t>P2016-2  G MOCHILA  CORO SINTEDICO JOGO TECIDO</t>
+  </si>
+  <si>
+    <t>39095029</t>
+  </si>
+  <si>
+    <t>21125</t>
+  </si>
+  <si>
+    <t>DS13454 TAPETE ANTIDERRAPANTE</t>
+  </si>
+  <si>
+    <t>57019000</t>
+  </si>
+  <si>
     <t>21447</t>
   </si>
   <si>
@@ -70,55 +157,46 @@
     <t>39169010</t>
   </si>
   <si>
-    <t>22594</t>
-  </si>
-  <si>
-    <t>MY-7327 MINI SOM ASTRONAUTA CX-60</t>
-  </si>
-  <si>
-    <t>85189010</t>
-  </si>
-  <si>
-    <t>25522</t>
-  </si>
-  <si>
-    <t>8805 ISQUEIRO  ELETRICO</t>
-  </si>
-  <si>
-    <t>85113020</t>
-  </si>
-  <si>
-    <t>26781</t>
-  </si>
-  <si>
-    <t>ST-06 SMART TAG BLEUTOOTH - CERIFICADO</t>
-  </si>
-  <si>
-    <t>85269100</t>
-  </si>
-  <si>
-    <t>26782</t>
-  </si>
-  <si>
-    <t>ST-05 SLING TAG- DISPOSITIVO LOCALIZADOR</t>
-  </si>
-  <si>
-    <t>28705</t>
-  </si>
-  <si>
-    <t>46257 IRRIGADOR ORAL</t>
-  </si>
-  <si>
-    <t>84248910</t>
-  </si>
-  <si>
-    <t>32041</t>
-  </si>
-  <si>
-    <t>NEW-215 - MODELADOR CORPORAL FEMININO EM POLIESTER E ELASTANO</t>
-  </si>
-  <si>
-    <t>62123000</t>
+    <t>22212</t>
+  </si>
+  <si>
+    <t>CA20155 CESTO DE PALHA QUADRADO G</t>
+  </si>
+  <si>
+    <t>46029000</t>
+  </si>
+  <si>
+    <t>22391</t>
+  </si>
+  <si>
+    <t>XL24152 CHAIRA 10'</t>
+  </si>
+  <si>
+    <t>82031090</t>
+  </si>
+  <si>
+    <t>22512</t>
+  </si>
+  <si>
+    <t>XL24151 CHAIRA 8' - 31 CM</t>
+  </si>
+  <si>
+    <t>26965</t>
+  </si>
+  <si>
+    <t>TOP7745 DISCO ABRASIVO P CORTE 115MM</t>
+  </si>
+  <si>
+    <t>68042219</t>
+  </si>
+  <si>
+    <t>28476</t>
+  </si>
+  <si>
+    <t>LB039047 - LENCO FEMININO CONFECCIONADO DE FIBRAS SINTETICAS</t>
+  </si>
+  <si>
+    <t>62143000</t>
   </si>
   <si>
     <t>33864</t>
@@ -137,81 +215,6 @@
   </si>
   <si>
     <t>84254990</t>
-  </si>
-  <si>
-    <t>39147</t>
-  </si>
-  <si>
-    <t>B39 BLUSA BRASIL AMARELA TAMANHO ÚNICO</t>
-  </si>
-  <si>
-    <t>61059000</t>
-  </si>
-  <si>
-    <t>39187</t>
-  </si>
-  <si>
-    <t>B13 BLUSA BRASIL VERDE TAMANHO ÚNICO</t>
-  </si>
-  <si>
-    <t>39188</t>
-  </si>
-  <si>
-    <t>B41 BLUSA BRASIL AMARELA TAM G</t>
-  </si>
-  <si>
-    <t>39189</t>
-  </si>
-  <si>
-    <t>B20 BLUSA BRASIL VERDE TAM G</t>
-  </si>
-  <si>
-    <t>39190</t>
-  </si>
-  <si>
-    <t>B15 BLUSA BRASIL BRANCA TAM G</t>
-  </si>
-  <si>
-    <t>39191</t>
-  </si>
-  <si>
-    <t>B-13 BLUSA BRASIL AZUL TAM G</t>
-  </si>
-  <si>
-    <t>39192</t>
-  </si>
-  <si>
-    <t>B19 BLUSA BRASIL BRANCA TAM M</t>
-  </si>
-  <si>
-    <t>39195</t>
-  </si>
-  <si>
-    <t>B28 BLUSA BRASIL VERDE TAM M</t>
-  </si>
-  <si>
-    <t>39196</t>
-  </si>
-  <si>
-    <t>B23 BLUSA BRASIL AZUL TAM M</t>
-  </si>
-  <si>
-    <t>18427</t>
-  </si>
-  <si>
-    <t>P2016-2  G MOCHILA  CORO SINTEDICO JOGO TECIDO</t>
-  </si>
-  <si>
-    <t>39095029</t>
-  </si>
-  <si>
-    <t>31403</t>
-  </si>
-  <si>
-    <t>LWJ-1953 KIT DE BROCAS ESCALONADAS EM ACO ACONDICIONADAS EM ESTOJO ORGANIZADOR</t>
-  </si>
-  <si>
-    <t>82075090</t>
   </si>
 </sst>
 </file>
@@ -588,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -627,7 +630,7 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -636,7 +639,7 @@
         <v>9</v>
       </c>
       <c r="F2">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -647,7 +650,7 @@
         <v>11</v>
       </c>
       <c r="C3">
-        <v>0.91</v>
+        <v>12.2</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
@@ -656,7 +659,7 @@
         <v>9</v>
       </c>
       <c r="F3">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -667,7 +670,7 @@
         <v>14</v>
       </c>
       <c r="C4">
-        <v>0.35</v>
+        <v>1.75</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
@@ -676,7 +679,7 @@
         <v>9</v>
       </c>
       <c r="F4">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -687,10 +690,10 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
@@ -701,16 +704,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
       <c r="C6">
-        <v>3.6</v>
+        <v>2.45</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E6" t="s">
         <v>9</v>
@@ -721,76 +724,76 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7">
+        <v>0.9</v>
+      </c>
+      <c r="D7" t="s">
         <v>22</v>
       </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7">
-        <v>1.45</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
-      </c>
       <c r="E7" t="s">
         <v>9</v>
       </c>
       <c r="F7">
-        <v>70</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>3.75</v>
+        <v>1.25</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
       </c>
       <c r="F8">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C9">
-        <v>3.75</v>
+        <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
         <v>9</v>
       </c>
       <c r="F9">
-        <v>100</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C10">
-        <v>3.4</v>
+        <v>14.4</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E10" t="s">
         <v>9</v>
@@ -801,93 +804,93 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11">
-        <v>8</v>
+        <v>0.55</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E11" t="s">
         <v>9</v>
       </c>
       <c r="F11">
-        <v>15</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C12">
-        <v>6.7</v>
+        <v>0.35</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E12" t="s">
         <v>9</v>
       </c>
       <c r="F12">
-        <v>10</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C13">
-        <v>14.5</v>
+        <v>2.99</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>3465</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C14">
-        <v>2.7</v>
+        <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E14" t="s">
         <v>9</v>
       </c>
       <c r="F14">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C15">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="D15" t="s">
         <v>44</v>
@@ -896,47 +899,47 @@
         <v>9</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16">
+        <v>0.5</v>
+      </c>
+      <c r="D16" t="s">
         <v>47</v>
       </c>
-      <c r="B16" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16">
-        <v>2.7</v>
-      </c>
-      <c r="D16" t="s">
-        <v>44</v>
-      </c>
       <c r="E16" t="s">
         <v>9</v>
       </c>
       <c r="F16">
-        <v>15</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" t="s">
         <v>49</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17">
+        <v>2.5</v>
+      </c>
+      <c r="D17" t="s">
         <v>50</v>
       </c>
-      <c r="C17">
-        <v>2.7</v>
-      </c>
-      <c r="D17" t="s">
-        <v>44</v>
-      </c>
       <c r="E17" t="s">
         <v>9</v>
       </c>
       <c r="F17">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -947,30 +950,30 @@
         <v>52</v>
       </c>
       <c r="C18">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="D18" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E18" t="s">
         <v>9</v>
       </c>
       <c r="F18">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19">
+        <v>2.05</v>
+      </c>
+      <c r="D19" t="s">
         <v>53</v>
-      </c>
-      <c r="B19" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19">
-        <v>2.7</v>
-      </c>
-      <c r="D19" t="s">
-        <v>44</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -981,16 +984,16 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C20">
-        <v>2.7</v>
+        <v>0.5</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
@@ -1001,82 +1004,62 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C21">
-        <v>2.2</v>
+        <v>1.55</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
       </c>
       <c r="F21">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C22">
-        <v>2.7</v>
+        <v>6.7</v>
       </c>
       <c r="D22" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
       </c>
       <c r="F22">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C23">
-        <v>39</v>
+        <v>14.5</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
       </c>
       <c r="F23">
         <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>64</v>
-      </c>
-      <c r="B24" t="s">
-        <v>65</v>
-      </c>
-      <c r="C24">
-        <v>4.6</v>
-      </c>
-      <c r="D24" t="s">
-        <v>66</v>
-      </c>
-      <c r="E24" t="s">
-        <v>9</v>
-      </c>
-      <c r="F24">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>